<commit_message>
feat: implement 7s repeat for instruction VO and idle prompts on pages G2 and T1
- Updated TAP_IN_SCENE to repeat the instruction VO after 7 seconds of inactivity on page G2, enhancing user engagement.
- Introduced a new mechanism to manage idle time, allowing the question to repeat after 7 seconds of silence, ensuring the child is prompted appropriately.
- Adjusted cue repeat timing for pages T2-T9 to 7 seconds, aligning with the new inactivity rule.
- Modified story_read_page.js to reflect the updated cue repeat logic, ensuring consistency across the application.
</commit_message>
<xml_diff>
--- a/HI02H04_L02_S01_HTML_Self_Review_Checklist_2026-10-12.xlsx
+++ b/HI02H04_L02_S01_HTML_Self_Review_Checklist_2026-10-12.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>What the lesson does (checked on the 12 Oct 2026 build)</t>
+          <t>What the lesson does (checked on the 12 Oct 2026 build, after the 7 s change)</t>
         </is>
       </c>
     </row>
@@ -821,25 +821,25 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Story pages T1–T9: the mic cue (pulse + «इस बटन पर टैप करिए और वाक्य पढ़िए।») repeats while nothing is tapped; all seven question pages: the question repeats (G3, I3, M1, M2 with the picture pop). None on the find page G2 (its lines escalate only on wrong taps), the car screens, the title or the end screen (no task waits there).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="27" customHeight="1">
+          <t>Story pages T1–T9: the mic cue (pulse + «इस बटन पर टैप करिए और वाक्य पढ़िए।») repeats while nothing is tapped; the find page G2 and all seven question pages: the question repeats (G3, I3, M1, M2 with the picture pop). None on the car screens, the title or the end screen (no task waits there).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1">
       <c r="A18" s="2" t="n"/>
       <c r="B18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Inactivity nudges are activated after 7 seconds. </t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>7 s on the seven question pages (quiet-and-free time, restarted by any tap or line). Story pages repeat after 4 s (T2–T9, as requested on 7 Oct) and 5 s on T1; G2 has no inactivity nudge.</t>
+          <t>7 s everywhere since the 12 Oct change: story pages T1–T9 repeat the cue 7 s after the previous cue (any tap restarts the count); G2 and the seven question pages repeat the question after 7 s of quiet-and-free time (not during a line, not after the third-miss hand). Measured 7.0–7.2 s.</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
         </is>
       </c>
       <c r="C62" s="10" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="63">
@@ -1577,7 +1577,7 @@
         </is>
       </c>
       <c r="C63" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
@@ -1597,10 +1597,10 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="27" customHeight="1">
+    <row r="67" ht="40.5" customHeight="1">
       <c r="B67" s="13" t="inlineStr">
         <is>
-          <t>Not matched: BGM already playing on the title screen (row 'The background music plays after the play button is tapped'); story-page nudges at 4–5 s and none on G2 (row 'Inactivity nudges are activated after 7 seconds'); first gate wording «चलिए, शुरू करें!» (row 'चलिए, शुरू करते हैं|').</t>
+          <t>Not matched: BGM already playing on the title screen (row 'The background music plays after the play button is tapped'); first gate wording «चलिए, शुरू करें!» (row 'चलिए, शुरू करते हैं|'). The 7 s inactivity row was a ✗ on the morning build (story pages 4–5 s, none on G2) and is a ✓ after the 12 Oct afternoon change.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor background music handling: update landing behavior to play on user interaction
- Modified bgm_duck.js to ensure background music only plays after the user taps the Play button on the title page, aligning with user request from 2026-10-12.
- Updated the card configuration in build.py to set 'landing' to False, preventing music from playing on the title page and ensuring it starts on the Play tap.
- Adjusted comments in both files for clarity regarding the new behavior and its implementation.
</commit_message>
<xml_diff>
--- a/HI02H04_L02_S01_HTML_Self_Review_Checklist_2026-10-12.xlsx
+++ b/HI02H04_L02_S01_HTML_Self_Review_Checklist_2026-10-12.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>What the lesson does (checked on the 12 Oct 2026 build, after the 7 s change)</t>
+          <t>What the lesson does (checked on the 12 Oct 2026 build, after the 7 s and music changes)</t>
         </is>
       </c>
     </row>
@@ -767,7 +767,7 @@
       <c r="C14" s="5" t="n"/>
       <c r="D14" s="2" t="n"/>
     </row>
-    <row r="15" ht="27" customHeight="1">
+    <row r="15" ht="40.5" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>General</t>
@@ -785,7 +785,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>bgm_standard_2 (Standard Background Music 2), ducked under every line (0.13 base / 0.03 while a line plays), from the title screen to M2; none on the end screen.</t>
+          <t>bgm_standard_2 (Standard Background Music 2), ducked under every line (0.13 base / 0.03 while a line plays), from the Play tap through the car finale; none on the title screen or the end screen.</t>
         </is>
       </c>
     </row>
@@ -796,14 +796,14 @@
           <t xml:space="preserve">The background music plays after the play button is tapped. </t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>The bed starts on the title screen itself — play() at 1.8 s together with the welcome line (card bgm.landing = true), i.e. before the Play tap wherever the browser allows autoplay. One flag (bgm.landing = false) would start it at the Play tap instead.</t>
+          <t>Since the 12 Oct change the title screen is silent (no bed under the welcome or a speaker-chip replay); the bed starts on the Play tap itself (36 ms after it), ducked under the first transition line, up to 0.13 in the quiet gap after it, and runs on through the lesson.</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
         </is>
       </c>
       <c r="C62" s="10" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="63">
@@ -1577,7 +1577,7 @@
         </is>
       </c>
       <c r="C63" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -1600,7 +1600,7 @@
     <row r="67" ht="40.5" customHeight="1">
       <c r="B67" s="13" t="inlineStr">
         <is>
-          <t>Not matched: BGM already playing on the title screen (row 'The background music plays after the play button is tapped'); first gate wording «चलिए, शुरू करें!» (row 'चलिए, शुरू करते हैं|'). The 7 s inactivity row was a ✗ on the morning build (story pages 4–5 s, none on G2) and is a ✓ after the 12 Oct afternoon change.</t>
+          <t>Not matched: first gate wording «चलिए, शुरू करें!» (row 'चलिए, शुरू करते हैं|'). Two rows were ✗ on the morning build and are ✓ after the 12 Oct afternoon changes: the 7 s inactivity rule (story pages were 4–5 s, G2 had none) and the music starting only after the Play tap (it used to start on the title screen).</t>
         </is>
       </c>
     </row>

</xml_diff>